<commit_message>
Singapore RT speaker: Alan Chow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
@@ -576,7 +576,7 @@
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>未確定事項の確認先（内閣府分は 9/30 確定: 林室長は英語で挨拶、肩書 Deputy Minister for Disaster Management, Cabinet Office of Japan、Gala 欠席。内閣府スケジュール 9/28 版〈10/1 受領〉: 28 日 RT Part 1 の日本発言＝中根補佐、SC 議長＝中根補佐、林室長は 13:10 SIDEX 視察→15:30 MHA〈バイ会談・MoC 署名〉→22:20 発、御手洗参事官は 28 日 MHA 同行・Gala 代理出席・29 日 RT Part 2／TS／Closing／Field Trip 出席・22:50 発、中根補佐は 29 日 RT Part 2／TS／Closing／SCDF パレード、青木補佐・起塚は日本パビリオン担当で 30 日 22:20 発）。ADRC＝評価フォーム（用意・URL/QR）、RT の質問方式、Co-Moderator の要否。Sylvia（SCDF/COSEM）＝シンガポールの RT 発言者の氏名・肩書、フィールドトリップのバス乗り場、パレードの時刻、Coffee Break の数量。ADRC 内部＝集合写真の対象範囲。</t>
+          <t>未確定事項の確認先（内閣府分は 9/30 確定: 林室長は英語で挨拶、肩書 Deputy Minister for Disaster Management, Cabinet Office of Japan、Gala 欠席。内閣府スケジュール 9/28 版〈10/1 受領〉: 28 日 RT Part 1 の日本発言＝中根補佐、SC 議長＝中根補佐、林室長は 13:10 SIDEX 視察→15:30 MHA〈バイ会談・MoC 署名〉→22:20 発、御手洗参事官は 28 日 MHA 同行・Gala 代理出席・29 日 RT Part 2／TS／Closing／Field Trip 出席・22:50 発、中根補佐は 29 日 RT Part 2／TS／Closing／SCDF パレード、青木補佐・起塚は日本パビリオン担当で 30 日 22:20 発）。ADRC＝評価フォーム（用意・URL/QR）、RT の質問方式、Co-Moderator の要否。Sylvia（SCDF/COSEM）＝フィールドトリップのバス乗り場、パレードの時刻、Coffee Break の数量。ADRC 内部＝集合写真の対象範囲。</t>
         </is>
       </c>
     </row>
@@ -2657,14 +2657,14 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Next, I would like to invite the delegation of Singapore. You have 5 minutes, please.
+          <t>Next, I would like to invite Mr Alan Chow, Director, Planning and Organisation Department, Singapore Civil Defence Force. You have 5 minutes, please.
 （ステートメント 5分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>10/8 Sylvia: シンガポールの発言者は SCDF の Director（ブリーフィングの音声では「Anancho, Director …」と聞こえ、氏名・肩書は未確認）【TBC・Sylvia に文字で確認】。Sylvia は本人に発言の準備を伝える。</t>
+          <t>シンガポールの発言者は Mr Alan Chow, Director, Planning &amp; Organisation Department, SCDF（10/8 ブリーフィングで Sylvia。音声は「Anancho, Director P&amp;O」）。Sylvia が本人に発言準備を伝える。</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Room is Peridot 204-206; fix scenario, note rework of power plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B15"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="2" max="2"/>
@@ -506,7 +506,7 @@
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>・会場: Peridot 201-203, Singapore EXPO。使用言語: 英語。Zoom Webinar による双方向ハイブリッド（オンライン登壇の可能性: UNDP・WMO＝未登録）。AI通訳（日本語）は神戸側が監視。
+          <t>・会場: Peridot 204-206, Singapore EXPO。使用言語: 英語。Zoom Webinar による双方向ハイブリッド（オンライン登壇の可能性: UNDP・WMO＝未登録）。AI通訳（日本語）は神戸側が監視。
 ・AI 翻訳＝ポケトークライブ（Sentio）。ホストは神戸（中村）が Zoom の音声を入力して運用する。参加者は QR（PPT 08 と卓上カード）を読み、自分の携帯や PC で翻訳言語を選んで読む。会場スクリーンへの字幕投影はしない。QR/URL は神戸が共有を開始した時点で発行されるので事前印刷はできない（共有開始直後に神戸が QR 画像を現地へ送り、現地でスライド貼付と案内カード印刷）。仕様（プレミアムプラン、pocketalk.jp/sentio/lineup・取扱説明書 10/1 確認）: 通訳の連続利用は 1 回 90 分、月の累計は無制限、共有可能人数 50 名、共有 URL/QR は共有開始から 6 時間で自動破棄。カンファレンスプランは連続無制限・URL 固定・50 名超も可（見積り制、リハーサル無償）。→ 運用: 通訳は 90 分ごとに藤本が再開（28 日 14:08 頃＝RT 13 番目の発言者の後、29 日 10:20 頃＝TS 発表 3 と 4 の間、11:40 頃＝閉会前）。共有 URL は本番用を 28 日 12:40、29 日 08:55 に開始する（08:00 の接続テストで開いた共有は必ず終了。6 時間で URL が破棄されるため、テストの共有をそのまま使うと 14:00 頃に切れる）。通訳を再開しても同じ共有 URL が維持されるかは神戸のリハーサルで検証（維持されるなら QR の再掲示は不要。されない場合は再開時に新 QR＝PPT 08b／16b を 20 秒表示し MC が再読込みを案内）。同時閲覧 50 名を超える見込み（日本語字幕の需要が多い場合）ならカンファレンスプランの見積りを取る。担当: 現地一次対応 藤本、設定 中村（神戸）。</t>
         </is>
       </c>
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
     <row r="2">
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Scenario_ACDR2026  Day 1 (Wed 28 Oct 2026)  ACDR Opening 12:45-13:00 / Roundtable Part 1 13:00-15:00   Venue: Peridot 201-203, Singapore EXPO</t>
+          <t>Scenario_ACDR2026  Day 1 (Wed 28 Oct 2026)  ACDR Opening 12:45-13:00 / Roundtable Part 1 13:00-15:00   Venue: Peridot 204-206, Singapore EXPO</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:P33"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3138,7 +3138,7 @@
     <row r="2">
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Scenario_ACDR2026  Day 2 (Thu 29 Oct 2026)  Roundtable Part 2 09:00-09:30 / Technical Session 09:30-11:30 / Summary &amp; Closing 11:45-12:00   Venue: Peridot 201-203</t>
+          <t>Scenario_ACDR2026  Day 2 (Thu 29 Oct 2026)  Roundtable Part 2 09:00-09:30 / Technical Session 09:30-11:30 / Summary &amp; Closing 11:45-12:00   Venue: Peridot 204-206</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Apply camera-in-U and room 204-206 to run sheet, scenario, packing list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_案1008.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="B1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="2" max="2"/>
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="B1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -763,7 +763,7 @@
         <is>
           <t>- PC（発表用・Zoom用）とスクリーン切替をAVオペと確認
 - 卓上マイク（U字14本＋教室列2本）、スタンド4、ハンド2、演台マイクの音出し
-- Zoom Webinar 起動（神戸: 中村）、ADRC 持込カメラ（Zoom 用、HDMI）の画角確認。2台目（U字パン）は未決
+- Zoom Webinar 起動（神戸: 中村）、カメラ 1 台（U 字の内側中央。業者カメラか ADRC カメラかは未決）の画角確認。電源・HDMI は AV 卓（前方右）から床に這わせて固定（約 12m）
 - AI通訳の日本語出力を神戸で確認
 - 名札・国旗プレートを配席表（0928）どおり配置</t>
         </is>
@@ -3107,7 +3107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="B1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5096,7 +5096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="B1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>

</xml_diff>